<commit_message>
L'avancement se teinte au lieu de se remplir
Google Sheets ne connaît pas les barres de données : à l'import, la barre
disparaissait et il ne restait que « 9/12 ». Or c'est en ligne que les
bénévoles regardent le tableur. Un dégradé à trois couleurs, lui, passe
dans les deux sens.

Il relie les trois teintes que le tableur emploie déjà : l'orange de
« Non traduit » à 0, le jaune d'« Ancienne version » au milieu, l'olive
d'« Enregistré » à 12. Aucun code couleur de plus à retenir.

Le compte, son format d'affichage et les treize autres règles ne bougent
pas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UK6pitX77pKQJxonxQtbux
</commit_message>
<xml_diff>
--- a/data_traduction.xlsx
+++ b/data_traduction.xlsx
@@ -1020,7 +1020,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Calculé tout seul, ne rien y écrire : le compte des 12 cases de la langue (6 traductions + 6 enregistrements), affiché « 9/12 ». Une « Ancienne version » vaut une demie, d'où les « 4,5/12 ». La barre de couleur remplit la cellule à proportion, pour voir l'avancement sans lire les chiffres.</t>
+          <t>Calculé tout seul, ne rien y écrire : le compte des 12 cases de la langue (6 traductions + 6 enregistrements), affiché « 9/12 ». Une « Ancienne version » vaut une demie, d'où les « 4,5/12 ». La cellule se teinte de l'orange au vert selon l'avancement, pour lire la colonne sans lire les chiffres.</t>
         </is>
       </c>
       <c r="C13" s="8" t="n"/>
@@ -50756,12 +50756,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G43">
-    <cfRule type="dataBar" priority="14">
-      <dataBar showValue="1">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
         <cfvo type="num" val="0"/>
+        <cfvo type="num" val="6"/>
         <cfvo type="num" val="12"/>
-        <color rgb="FF9DA679"/>
-      </dataBar>
+        <color rgb="FFF4BB8F"/>
+        <color rgb="FFF9EFA8"/>
+        <color rgb="FFC4C9AE"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">

</xml_diff>